<commit_message>
fix: hapus teks transfer dan perbaiki teks kwitansi cukup sampai di UP Taman Margasatwa Ragunan serta perbaiki terbilang
</commit_message>
<xml_diff>
--- a/public/kwitansi rombongan.xlsx
+++ b/public/kwitansi rombongan.xlsx
@@ -1,32 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\.gemini\antigravity-ide\scratch\sistem-informasi-ragunan\public\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6D16A73-7C45-4E93-8792-A95D9B80AABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="1068" yWindow="1140" windowWidth="17280" windowHeight="8832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1068" yWindow="1140" windowWidth="17280" windowHeight="8832"/>
   </bookViews>
   <sheets>
-    <sheet name="kwitansi kosong" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="kwitansi kosong" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
@@ -36,13 +19,36 @@
     <t xml:space="preserve">Sudah terima dari </t>
   </si>
   <si>
+    <r>
+      <t>&lt;&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <color theme="1"/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+      </rPr>
+      <t>Nama Penyewa&gt;&gt;</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">Terbilang </t>
+  </si>
+  <si>
+    <t>&lt;&lt;Terbilang&gt;&gt;</t>
   </si>
   <si>
     <t>Untuk pembayaran</t>
   </si>
   <si>
-    <t>di UP Taman Margasatwa Ragunan melalui transfer &lt;&lt;Transfer&gt;&gt; dengan No.ref &lt;&lt;reff&gt;&gt;</t>
+    <t xml:space="preserve">kegiatan &lt;&lt;Kegiatan&gt;&gt; di lokasi &lt;&lt;Lokasi Sewa&gt;&gt; </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> pada tanggal &lt;&lt;Tanggal Sewa&gt;&gt;</t>
+  </si>
+  <si>
+    <t>di UP Taman Margasatwa Ragunan</t>
   </si>
   <si>
     <t>Jakarta, &lt;&lt;tanggal&gt;&gt; &lt;&lt;bulan&gt;&gt; &lt;&lt;tahun&gt;&gt;</t>
@@ -56,80 +62,58 @@
   <si>
     <t xml:space="preserve"> Rupiah</t>
   </si>
-  <si>
-    <r>
-      <t>&lt;&lt;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-      </rPr>
-      <t>Nama Penyewa&gt;&gt;</t>
-    </r>
-  </si>
-  <si>
-    <t>&lt;&lt;Terbilang&gt;&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> pada tanggal &lt;&lt;Tanggal Sewa&gt;&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kegiatan &lt;&lt;Kegiatan&gt;&gt; di lokasi &lt;&lt;Lokasi Sewa&gt;&gt; </t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* (#,##0);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* (#,##0.00);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* (#,##0);_(* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="&quot;Rp&quot;#,##0;[Red]&quot;Rp&quot;#,##0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <color theme="1"/>
+      <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <i/>
+      <color theme="1"/>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <color theme="1"/>
+      <scheme val="minor"/>
       <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
       <scheme val="minor"/>
+      <sz val="10"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
+      <color theme="0"/>
+      <scheme val="minor"/>
       <sz val="10"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="1"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -153,7 +137,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -165,24 +149,6 @@
       <left style="thin">
         <color rgb="FF000000"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color rgb="FF000000"/>
@@ -221,44 +187,9 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -276,70 +207,9 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top/>
       <bottom style="dotted">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="dotted">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="double">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="double">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="double">
         <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
@@ -377,15 +247,6 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color rgb="FF000000"/>
       </right>
@@ -399,40 +260,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -444,50 +294,39 @@
     <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment textRotation="255"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="167" fontId="2" fillId="2" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,7 +346,7 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>38100</xdr:colOff>
@@ -517,14 +356,16 @@
     <xdr:ext cx="1162050" cy="3057525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="image3.png" title="Image">
+        <xdr:cNvPr id="1" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
@@ -533,15 +374,18 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
+    <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>114300</xdr:colOff>
@@ -551,14 +395,16 @@
     <xdr:ext cx="228600" cy="876300"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="image1.png" title="Gambar">
+        <xdr:cNvPr id="2" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print"/>
@@ -567,15 +413,18 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
+    <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
+  <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>142875</xdr:colOff>
@@ -585,14 +434,16 @@
     <xdr:ext cx="628650" cy="752475"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="image2.png" title="Gambar">
+        <xdr:cNvPr id="3" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
         <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print"/>
@@ -601,19 +452,18 @@
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData fLocksWithSheet="0"/>
+    <xdr:clientData/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -813,9 +663,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:X1007"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25" defaultColWidth="12.6640625"/>
   <cols>
     <col min="1" max="3" width="8.6640625" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
@@ -833,526 +683,526 @@
     <col min="19" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="3" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
-      <c r="R5" s="5"/>
-    </row>
-    <row r="6" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="12"/>
-    </row>
-    <row r="7" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="12"/>
-    </row>
-    <row r="8" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11" t="s">
+      <c r="R5" s="4"/>
+    </row>
+    <row r="6" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="6"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="6"/>
+      <c r="Q6" s="6"/>
+      <c r="R6" s="8"/>
+    </row>
+    <row r="7" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="K7" s="6"/>
+      <c r="L7" s="6"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="6"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="6"/>
+      <c r="Q7" s="6"/>
+      <c r="R7" s="8"/>
+    </row>
+    <row r="8" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="15" t="s">
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="6"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="6"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="8"/>
+    </row>
+    <row r="9" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="8"/>
+    </row>
+    <row r="10" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="5"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="14"/>
+      <c r="L10" s="14"/>
+      <c r="M10" s="14"/>
+      <c r="N10" s="14"/>
+      <c r="O10" s="14"/>
+      <c r="P10" s="14"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="8"/>
+    </row>
+    <row r="11" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="5"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" s="14"/>
+      <c r="I11" s="14"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="14"/>
+      <c r="L11" s="14"/>
+      <c r="M11" s="14"/>
+      <c r="N11" s="14"/>
+      <c r="O11" s="14"/>
+      <c r="P11" s="14"/>
+      <c r="Q11" s="15"/>
+      <c r="R11" s="8"/>
+    </row>
+    <row r="12" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="5"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="14"/>
+      <c r="I12" s="14"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="14"/>
+      <c r="L12" s="14"/>
+      <c r="M12" s="14"/>
+      <c r="N12" s="14"/>
+      <c r="O12" s="14"/>
+      <c r="P12" s="14"/>
+      <c r="Q12" s="15"/>
+      <c r="R12" s="8"/>
+    </row>
+    <row r="13" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="8"/>
+    </row>
+    <row r="14" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="18"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="8"/>
+    </row>
+    <row r="15" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="6"/>
+      <c r="M15" s="19"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="8"/>
+    </row>
+    <row r="16" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="16"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="6"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="19"/>
+      <c r="P16" s="20"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="8"/>
+    </row>
+    <row r="17" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A17" s="5"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="6"/>
+      <c r="M17" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="12"/>
-    </row>
-    <row r="9" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11" t="s">
-        <v>1</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="17" t="s">
+      <c r="N17" s="23"/>
+      <c r="O17" s="23"/>
+      <c r="P17" s="23"/>
+      <c r="R17" s="8"/>
+    </row>
+    <row r="18" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A18" s="5"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="7"/>
+      <c r="M18" s="7"/>
+      <c r="N18" s="7"/>
+      <c r="O18" s="24"/>
+      <c r="P18" s="7"/>
+      <c r="Q18" s="18"/>
+      <c r="R18" s="8"/>
+    </row>
+    <row r="19" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A19" s="5"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="7"/>
+      <c r="M19" s="7"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="24"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="18"/>
+      <c r="R19" s="8"/>
+    </row>
+    <row r="20" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A20" s="5"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="7"/>
+      <c r="M20" s="7"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="25"/>
+      <c r="Q20" s="18"/>
+      <c r="R20" s="8"/>
+    </row>
+    <row r="21" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="16"/>
-      <c r="K9" s="16"/>
-      <c r="L9" s="16"/>
-      <c r="M9" s="16"/>
-      <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
-      <c r="P9" s="16"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="18"/>
-    </row>
-    <row r="10" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="21"/>
-      <c r="I10" s="21"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="22"/>
-      <c r="R10" s="12"/>
-    </row>
-    <row r="11" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="20" t="s">
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="7"/>
+      <c r="M21" s="7"/>
+      <c r="N21" s="7"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="28"/>
+      <c r="Q21" s="18"/>
+      <c r="R21" s="8"/>
+    </row>
+    <row r="22" ht="45.75" customHeight="1" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+      <c r="J22" s="31"/>
+      <c r="K22" s="31"/>
+      <c r="L22" s="31"/>
+      <c r="M22" s="31"/>
+      <c r="N22" s="31"/>
+      <c r="O22" s="31"/>
+      <c r="P22" s="32"/>
+      <c r="Q22" s="31"/>
+      <c r="R22" s="33"/>
+      <c r="X22" s="34"/>
+    </row>
+    <row r="23" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="7"/>
+      <c r="M23" s="7"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="7"/>
+      <c r="P23" s="28"/>
+      <c r="Q23" s="7"/>
+      <c r="R23" s="6"/>
+    </row>
+    <row r="24" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="7"/>
+      <c r="M24" s="7"/>
+      <c r="N24" s="7"/>
+      <c r="O24" s="7"/>
+      <c r="P24" s="28"/>
+      <c r="Q24" s="7"/>
+      <c r="R24" s="6"/>
+    </row>
+    <row r="25" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="7"/>
+      <c r="N25" s="7"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="28"/>
+      <c r="Q25" s="7"/>
+      <c r="R25" s="6"/>
+    </row>
+    <row r="26" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="7"/>
+      <c r="N26" s="7"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="28"/>
+      <c r="Q26" s="7"/>
+      <c r="R26" s="6"/>
+    </row>
+    <row r="27" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="7"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="28"/>
+      <c r="Q27" s="7"/>
+      <c r="R27" s="6"/>
+    </row>
+    <row r="28" ht="12.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="7"/>
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="7"/>
+      <c r="N28" s="7"/>
+      <c r="O28" s="7"/>
+      <c r="P28" s="28"/>
+      <c r="Q28" s="7"/>
+      <c r="R28" s="6"/>
+    </row>
+    <row r="29" ht="12.75" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="7"/>
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="7"/>
+      <c r="L29" s="7"/>
+      <c r="M29" s="7"/>
+      <c r="N29" s="7"/>
+      <c r="O29" s="7"/>
+      <c r="P29" s="28"/>
+      <c r="Q29" s="7"/>
+      <c r="R29" s="6"/>
+      <c r="U29" s="35"/>
+    </row>
+    <row r="30" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" ht="12.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="H11" s="21"/>
-      <c r="I11" s="21"/>
-      <c r="J11" s="21"/>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="21"/>
-      <c r="N11" s="21"/>
-      <c r="O11" s="21"/>
-      <c r="P11" s="21"/>
-      <c r="Q11" s="22"/>
-      <c r="R11" s="12"/>
-    </row>
-    <row r="12" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="21"/>
-      <c r="L12" s="21"/>
-      <c r="M12" s="21"/>
-      <c r="N12" s="21"/>
-      <c r="O12" s="21"/>
-      <c r="P12" s="21"/>
-      <c r="Q12" s="23"/>
-      <c r="R12" s="12"/>
-    </row>
-    <row r="13" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="12"/>
-    </row>
-    <row r="14" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="24"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="25"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="27"/>
-      <c r="L14" s="8"/>
-      <c r="M14" s="28"/>
-      <c r="N14" s="28"/>
-      <c r="O14" s="28"/>
-      <c r="P14" s="28"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="12"/>
-    </row>
-    <row r="15" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="28"/>
-      <c r="N15" s="8"/>
-      <c r="O15" s="28"/>
-      <c r="P15" s="29"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="12"/>
-    </row>
-    <row r="16" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="28"/>
-      <c r="N16" s="8"/>
-      <c r="O16" s="28"/>
-      <c r="P16" s="29"/>
-      <c r="Q16" s="30"/>
-      <c r="R16" s="12"/>
-    </row>
-    <row r="17" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="31"/>
-      <c r="J17" s="31"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="47" t="s">
-        <v>4</v>
-      </c>
-      <c r="N17" s="48"/>
-      <c r="O17" s="48"/>
-      <c r="P17" s="48"/>
-      <c r="R17" s="18"/>
-    </row>
-    <row r="18" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10"/>
-      <c r="O18" s="32"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="33"/>
-      <c r="R18" s="12"/>
-    </row>
-    <row r="19" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="6"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="10"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="32"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="34"/>
-      <c r="R19" s="12"/>
-    </row>
-    <row r="20" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="6"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="35"/>
-      <c r="Q20" s="34"/>
-      <c r="R20" s="12"/>
-    </row>
-    <row r="21" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="6"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="49" t="s">
-        <v>5</v>
-      </c>
-      <c r="E21" s="50"/>
-      <c r="F21" s="50"/>
-      <c r="G21" s="51"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="36"/>
-      <c r="Q21" s="34"/>
-      <c r="R21" s="12"/>
-    </row>
-    <row r="22" spans="1:24" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="37"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="38"/>
-      <c r="H22" s="39"/>
-      <c r="I22" s="39"/>
-      <c r="J22" s="39"/>
-      <c r="K22" s="39"/>
-      <c r="L22" s="39"/>
-      <c r="M22" s="39"/>
-      <c r="N22" s="39"/>
-      <c r="O22" s="39"/>
-      <c r="P22" s="40"/>
-      <c r="Q22" s="39"/>
-      <c r="R22" s="41"/>
-      <c r="X22" s="42"/>
-    </row>
-    <row r="23" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="10"/>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10"/>
-      <c r="O23" s="10"/>
-      <c r="P23" s="43"/>
-      <c r="Q23" s="10"/>
-      <c r="R23" s="8"/>
-    </row>
-    <row r="24" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="43"/>
-      <c r="Q24" s="10"/>
-      <c r="R24" s="8"/>
-    </row>
-    <row r="25" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="10"/>
-      <c r="M25" s="10"/>
-      <c r="N25" s="10"/>
-      <c r="O25" s="10"/>
-      <c r="P25" s="43"/>
-      <c r="Q25" s="10"/>
-      <c r="R25" s="8"/>
-    </row>
-    <row r="26" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10"/>
-      <c r="L26" s="10"/>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10"/>
-      <c r="O26" s="10"/>
-      <c r="P26" s="43"/>
-      <c r="Q26" s="10"/>
-      <c r="R26" s="8"/>
-    </row>
-    <row r="27" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="10"/>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10"/>
-      <c r="L27" s="10"/>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10"/>
-      <c r="O27" s="10"/>
-      <c r="P27" s="43"/>
-      <c r="Q27" s="10"/>
-      <c r="R27" s="8"/>
-    </row>
-    <row r="28" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="10"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10"/>
-      <c r="L28" s="10"/>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10"/>
-      <c r="O28" s="10"/>
-      <c r="P28" s="43"/>
-      <c r="Q28" s="10"/>
-      <c r="R28" s="8"/>
-    </row>
-    <row r="29" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="43"/>
-      <c r="Q29" s="10"/>
-      <c r="R29" s="8"/>
-      <c r="U29" s="44"/>
-    </row>
-    <row r="30" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="45" t="s">
-        <v>6</v>
-      </c>
-      <c r="K31" s="46"/>
-    </row>
-    <row r="32" spans="1:24" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="45" t="s">
-        <v>7</v>
+      <c r="K31" s="37"/>
+    </row>
+    <row r="32" ht="12.75" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="36" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="33" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2336,7 +2186,7 @@
     <mergeCell ref="D21:G21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="5" orientation="landscape"/>
+  <pageSetup paperSize="5" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>